<commit_message>
Rental Agreement day 5 updated branch push
</commit_message>
<xml_diff>
--- a/src/test/resources/Landlord_Tenant_details.xlsx
+++ b/src/test/resources/Landlord_Tenant_details.xlsx
@@ -3,19 +3,15 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cc811f361f3f8b4c/Desktop/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{D3BF3DA1-B7F7-42FB-80EB-903A575D0FE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AE6D041B-1E16-4C91-9E70-097573FBE853}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{FF0C331B-4110-4D74-B848-B22FCEF342F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B07F5926-60FD-4560-A73A-4B3022D93537}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>

</xml_diff>

<commit_message>
Resolved conflicts while meging master with Rental Module
</commit_message>
<xml_diff>
--- a/src/test/resources/Landlord_Tenant_details.xlsx
+++ b/src/test/resources/Landlord_Tenant_details.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{FF0C331B-4110-4D74-B848-B22FCEF342F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{3E6C1910-A70E-43EE-8869-CD6374DCE64A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B07F5926-60FD-4560-A73A-4B3022D93537}"/>
   </bookViews>
@@ -11,21 +11,10 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1"/>
+  <oleSize ref="A1:K32"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>

</xml_diff>